<commit_message>
RELEASE WITH TRACK PANT SHOPSY
</commit_message>
<xml_diff>
--- a/Full-LC-AUTO/dist/release/Full-LC-AUTO/data inputs/track_pant/Product-Description-inputs.xlsx
+++ b/Full-LC-AUTO/dist/release/Full-LC-AUTO/data inputs/track_pant/Product-Description-inputs.xlsx
@@ -1,11 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_E83AB7BEEC67F4F3CE483C7539646D63E753C1E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Track Pant Product Inputs" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Track Pant Field Guide" state="visible" r:id="rId5"/>
+    <sheet name="Track Pant Product Inputs" sheetId="1" r:id="rId1"/>
+    <sheet name="Track Pant Field Guide" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -116,17 +120,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -490,16 +496,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="11" width="18" customWidth="1"/>
-    <col min="12" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="12" max="24" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -534,7 +540,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -569,7 +575,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -604,7 +610,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -639,7 +645,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -676,23 +682,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="42.142857142857146" customWidth="1"/>
-    <col min="5" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="4" max="4" width="42.109375" customWidth="1"/>
+    <col min="5" max="24" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -706,7 +712,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -720,7 +726,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -734,7 +740,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -748,7 +754,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -762,7 +768,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -776,7 +782,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -790,7 +796,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -804,7 +810,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -818,7 +824,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -834,6 +840,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>